<commit_message>
dp on strings completed
</commit_message>
<xml_diff>
--- a/Strivers List + other Problems.xlsx
+++ b/Strivers List + other Problems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DSA Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973D696C-43F2-4D62-AE7F-A38373FD591A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38BAA385-F0B4-4242-B3B4-DF67A801B55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12601,7 +12601,7 @@
     <row r="275" spans="1:25" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A275" s="57"/>
       <c r="B275" s="50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C275" s="2">
         <v>24</v>

</xml_diff>

<commit_message>
DAY 1 lc practice
</commit_message>
<xml_diff>
--- a/Strivers List + other Problems.xlsx
+++ b/Strivers List + other Problems.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DSA Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38BAA385-F0B4-4242-B3B4-DF67A801B55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D5C601-7BE4-47CA-A254-5DD7D6EA6664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1838,7 +1838,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2011,6 +2011,7 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -8511,7 +8512,7 @@
     <row r="167" spans="1:25" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A167" s="62"/>
       <c r="B167" s="50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C167" s="30">
         <v>16</v>
@@ -10649,7 +10650,7 @@
     <row r="223" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A223" s="57"/>
       <c r="B223" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C223" s="2">
         <v>12</v>
@@ -10686,7 +10687,7 @@
     <row r="224" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A224" s="57"/>
       <c r="B224" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C224" s="2">
         <v>13</v>
@@ -10723,7 +10724,7 @@
     <row r="225" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A225" s="57"/>
       <c r="B225" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C225" s="2">
         <v>14</v>
@@ -10760,7 +10761,7 @@
     <row r="226" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A226" s="57"/>
       <c r="B226" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C226" s="2">
         <v>15</v>
@@ -10799,7 +10800,7 @@
     <row r="227" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A227" s="57"/>
       <c r="B227" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C227" s="2">
         <v>16</v>
@@ -10838,7 +10839,7 @@
     <row r="228" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A228" s="57"/>
       <c r="B228" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C228" s="2">
         <v>17</v>
@@ -10875,7 +10876,7 @@
     <row r="229" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A229" s="57"/>
       <c r="B229" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C229" s="2">
         <v>18</v>
@@ -11105,7 +11106,7 @@
     <row r="235" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A235" s="57"/>
       <c r="B235" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C235" s="2">
         <v>24</v>
@@ -11181,7 +11182,7 @@
     <row r="237" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A237" s="57"/>
       <c r="B237" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C237" s="2">
         <v>26</v>
@@ -11218,7 +11219,7 @@
     <row r="238" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A238" s="57"/>
       <c r="B238" s="50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C238" s="2">
         <v>27</v>
@@ -11671,9 +11672,9 @@
       <c r="X249" s="1"/>
       <c r="Y249" s="1"/>
     </row>
-    <row r="250" spans="1:25" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:25" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A250" s="1"/>
-      <c r="B250" s="1"/>
+      <c r="B250" s="68"/>
       <c r="C250" s="1"/>
       <c r="D250" s="1"/>
       <c r="E250" s="3"/>
@@ -11698,9 +11699,9 @@
       <c r="X250" s="1"/>
       <c r="Y250" s="1"/>
     </row>
-    <row r="251" spans="1:25" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:25" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A251" s="1"/>
-      <c r="B251" s="1"/>
+      <c r="B251" s="68"/>
       <c r="C251" s="1"/>
       <c r="D251" s="1"/>
       <c r="E251" s="3"/>
@@ -12718,7 +12719,7 @@
     <row r="278" spans="1:25" ht="15" x14ac:dyDescent="0.35">
       <c r="A278" s="57"/>
       <c r="B278" s="50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C278" s="2">
         <v>27</v>

</xml_diff>